<commit_message>
Refactor course title JSON files
</commit_message>
<xml_diff>
--- a/client/assets/final_sose_243.xlsx
+++ b/client/assets/final_sose_243.xlsx
@@ -2913,13 +2913,13 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -2980,10 +2980,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3300,7 +3300,7 @@
     <col min="5" max="5" style="9" width="9.43357142857143" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="9" width="17.290714285714284" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="9" width="20.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="8" width="26.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="8" width="140.71928571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -6293,7 +6293,7 @@
         <v>277</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="46.5">
       <c r="A116" s="4" t="s">
         <v>8</v>
       </c>
@@ -6319,7 +6319,7 @@
         <v>280</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="33">
       <c r="A117" s="4" t="s">
         <v>20</v>
       </c>
@@ -6345,7 +6345,7 @@
         <v>283</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="60">
       <c r="A118" s="4" t="s">
         <v>20</v>
       </c>
@@ -6371,7 +6371,7 @@
         <v>284</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="33">
       <c r="A119" s="4" t="s">
         <v>20</v>
       </c>
@@ -6397,7 +6397,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="60">
       <c r="A120" s="4" t="s">
         <v>20</v>
       </c>
@@ -6423,7 +6423,7 @@
         <v>290</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="60">
       <c r="A121" s="4" t="s">
         <v>8</v>
       </c>
@@ -6449,7 +6449,7 @@
         <v>291</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="60">
       <c r="A122" s="4" t="s">
         <v>8</v>
       </c>
@@ -6475,7 +6475,7 @@
         <v>292</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="60">
       <c r="A123" s="4" t="s">
         <v>8</v>
       </c>
@@ -6501,7 +6501,7 @@
         <v>293</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="60">
       <c r="A124" s="4" t="s">
         <v>8</v>
       </c>
@@ -6527,7 +6527,7 @@
         <v>294</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="60">
       <c r="A125" s="4" t="s">
         <v>8</v>
       </c>
@@ -6553,7 +6553,7 @@
         <v>295</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="60">
       <c r="A126" s="4" t="s">
         <v>8</v>
       </c>
@@ -6579,7 +6579,7 @@
         <v>296</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="60">
       <c r="A127" s="4" t="s">
         <v>8</v>
       </c>
@@ -6605,7 +6605,7 @@
         <v>297</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="60">
       <c r="A128" s="4" t="s">
         <v>8</v>
       </c>
@@ -6631,7 +6631,7 @@
         <v>299</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="60">
       <c r="A129" s="4" t="s">
         <v>8</v>
       </c>
@@ -6657,7 +6657,7 @@
         <v>301</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="46.5">
       <c r="A130" s="4" t="s">
         <v>8</v>
       </c>
@@ -6683,7 +6683,7 @@
         <v>305</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="46.5">
       <c r="A131" s="4" t="s">
         <v>8</v>
       </c>
@@ -6709,7 +6709,7 @@
         <v>307</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="46.5">
       <c r="A132" s="4" t="s">
         <v>8</v>
       </c>
@@ -6735,7 +6735,7 @@
         <v>308</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="46.5">
       <c r="A133" s="4" t="s">
         <v>8</v>
       </c>
@@ -6761,7 +6761,7 @@
         <v>311</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="33">
       <c r="A134" s="4" t="s">
         <v>20</v>
       </c>
@@ -6787,7 +6787,7 @@
         <v>314</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="60">
       <c r="A135" s="4" t="s">
         <v>20</v>
       </c>
@@ -6813,7 +6813,7 @@
         <v>316</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="33">
       <c r="A136" s="4" t="s">
         <v>20</v>
       </c>
@@ -6839,7 +6839,7 @@
         <v>317</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="33">
       <c r="A137" s="4" t="s">
         <v>20</v>
       </c>
@@ -6865,7 +6865,7 @@
         <v>320</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="60">
       <c r="A138" s="4" t="s">
         <v>8</v>
       </c>
@@ -6891,7 +6891,7 @@
         <v>324</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="46.5">
       <c r="A139" s="4" t="s">
         <v>8</v>
       </c>
@@ -6917,7 +6917,7 @@
         <v>325</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="33">
       <c r="A140" s="4" t="s">
         <v>20</v>
       </c>
@@ -6943,7 +6943,7 @@
         <v>329</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="33">
       <c r="A141" s="4" t="s">
         <v>8</v>
       </c>
@@ -6969,7 +6969,7 @@
         <v>333</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="46.5">
       <c r="A142" s="4" t="s">
         <v>20</v>
       </c>
@@ -6995,7 +6995,7 @@
         <v>337</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="60">
       <c r="A143" s="4" t="s">
         <v>20</v>
       </c>
@@ -7021,7 +7021,7 @@
         <v>339</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="33">
       <c r="A144" s="4" t="s">
         <v>8</v>
       </c>
@@ -7047,7 +7047,7 @@
         <v>343</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="33">
       <c r="A145" s="4" t="s">
         <v>8</v>
       </c>
@@ -7073,7 +7073,7 @@
         <v>344</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="60">
       <c r="A146" s="4" t="s">
         <v>8</v>
       </c>
@@ -7099,7 +7099,7 @@
         <v>345</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="60">
       <c r="A147" s="4" t="s">
         <v>8</v>
       </c>
@@ -7125,7 +7125,7 @@
         <v>346</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="60">
       <c r="A148" s="4" t="s">
         <v>8</v>
       </c>

</xml_diff>